<commit_message>
Remove people's names from the site, playbook, and QA workbook
Sources now describe sessions by role (HCM, costing, payroll SME sessions;
HCM training sessions 1 and 2). Drop the stale walkthrough note on the weekly
time card check. Leave courses refer to the Leave SME. Blur the remaining
name, initials, and profile photo in the UKG screenshots.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WqfFtE1Qb9uN7QDcn19AvE
</commit_message>
<xml_diff>
--- a/docs/HCM_Academy_QA_Review.xlsx
+++ b/docs/HCM_Academy_QA_Review.xlsx
@@ -9663,13 +9663,13 @@
       <c r="K56" s="8" t="inlineStr">
         <is>
           <t>- Which Oracle absence types Vanderbilt uses for FMLA, TMLA (TPLA), and FMLA running at the same time as state leave, and who enters intermittent occurrences, must be confirmed.
-- Vanderbilt's leave process is pending review by Sheila, the Leave SME.
+- Vanderbilt's leave process is pending review by the Leave SME.
 - Oracle absence types Vanderbilt uses for FMLA, TMLA/TPLA, and concurrent FMLA and state leave
 - Who enters intermittent occurrences (HCM, employee, or Leave team) and how often
 - Whether FMLA is tracked in hours or days at Vanderbilt and which 12-month period method is used
 - Current TPLA eligibility rules and leave length in T.C.A. 4-21-408 (confirm with Leave SME or legal)
 - Whether a continuous FMLA/TMLA leave also requires a leave status change in Change Assignment
-- Sheila (Leave SME) review of the full FMLA/TMLA process</t>
+- The Leave SME (Leave SME) review of the full FMLA/TMLA process</t>
         </is>
       </c>
       <c r="L56" s="6" t="inlineStr"/>
@@ -9792,12 +9792,12 @@
       <c r="K58" s="8" t="inlineStr">
         <is>
           <t>- Vanderbilt's approval routing for each absence type (who approves, whether HR or the Leave team is in the chain, what happens if an approver does not act) must be confirmed.
-- Vanderbilt's leave process is pending review by Sheila, the Leave SME.
+- Vanderbilt's leave process is pending review by the Leave SME.
 - Approval routing for each Vanderbilt absence type (approvers, Leave team involvement)
 - Whether absence approvals expire or escalate, and the action on expiry
 - Whether HCMs can see and act on requests for their area in the notifications bell
 - Whether withdrawals of approved absences require approval at Vanderbilt
-- Sheila (Leave SME) review of the full workflow</t>
+- The Leave SME (Leave SME) review of the full workflow</t>
         </is>
       </c>
       <c r="L58" s="6" t="inlineStr"/>
@@ -9865,11 +9865,11 @@
       <c r="K59" s="8" t="inlineStr">
         <is>
           <t>- Which quick actions HCMs see under Our Workforce, and whether HCMs approve exempt time off or only managers do, must be confirmed on screen.
-- Vanderbilt's leave process is pending review by Sheila, the Leave SME.
+- Vanderbilt's leave process is pending review by the Leave SME.
 - Which absence quick actions (Add Absence, Existing Absences, Absence Balance) HCMs see under Our Workforce &gt; Quick Actions
 - Absence types and plans available to exempt employees (vacation, sick, etc.)
 - Whether exempt time off can be entered in partial days or hours
-- Sheila (Leave SME) review of the full process</t>
+- The Leave SME (Leave SME) review of the full process</t>
         </is>
       </c>
       <c r="L59" s="6" t="inlineStr"/>

</xml_diff>